<commit_message>
Treat Quad Pro Max as live, not superseded
Quad Pro Max (240W, 1.5m) and the new Quad Pro Black (100W, 1.2m) are
different spec tiers that coexist rather than one replacing the other, and
Max is still selling at DRR 12. Running it down to a 15-day bridge was
wrong.

Max now takes the normal 35-day cap like any established SKU: ships 60 of
its 72 open units, landing at exactly 35 days. Only old GIGA and Click Slim
remain on run-down, as their successors genuinely supersede them.

Ship 4,281u (Rs 74.7L), up 60 units.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N5QckZ42nw4ueLobVZghMn
</commit_message>
<xml_diff>
--- a/analysis/cocoblu-supply-2026-09-04/Cocoblu_Supply_Plan_v3_ISK3.xlsx
+++ b/analysis/cocoblu-supply-2026-09-04/Cocoblu_Supply_Plan_v3_ISK3.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'0_Summary'!$A$1:$B$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1_Dispatch by PO'!$A$1:$F$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2_Dispatch lines'!$A$1:$N$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2_Dispatch lines'!$A$1:$N$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3_SKU plan 35d'!$A$1:$S$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4_Franchise cap'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5_Ask Amazon for PO'!$A$1:$K$7</definedName>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4221</v>
+        <v>4281</v>
       </c>
     </row>
     <row r="8">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7439495</v>
+        <v>7469978</v>
       </c>
     </row>
     <row r="9">
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9679</v>
+        <v>9619</v>
       </c>
     </row>
     <row r="10">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12">
@@ -695,10 +695,10 @@
         <v>46285</v>
       </c>
       <c r="E2" t="n">
-        <v>1566</v>
+        <v>1626</v>
       </c>
       <c r="F2" t="n">
-        <v>3206813</v>
+        <v>3237296</v>
       </c>
     </row>
     <row r="3">
@@ -845,7 +845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2397,50 +2397,50 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>5OF8HBIC</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>46237</v>
+        <v>46244</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>B0DPHR4FG7</t>
+          <t>B0D8443PTW</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>PBLUCIDWHT</t>
+          <t>QUADPROMAXBLK</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Stuffcool Lucid 15W Smallest Magnetic Wireless Powerbank 5000Mah Battery Capacity for iPhone 16</t>
+          <t>Stuffcool Quad Pro Max 4 in 1 Metal Braided Cable 1.5m 240W Rugged e-Marker chip gold plated co</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>942.96</v>
+        <v>508.05</v>
       </c>
       <c r="G29" t="n">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="H29" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="I29" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>46237</v>
+        <v>46244</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>46266</v>
+        <v>46285</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>46270</v>
+        <v>46289</v>
       </c>
       <c r="M29" t="n">
-        <v>28289</v>
+        <v>30483</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -2459,30 +2459,30 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>B0FT2VNW5H</t>
+          <t>B0DPHR4FG7</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>WCZENO30WWHT</t>
+          <t>PBLUCIDWHT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Stuffcool Zeno 30W GaN Type C Fast Charger Retractable Cable 75cm PD PPS iPhone Pixel Samsung S</t>
+          <t>Stuffcool Lucid 15W Smallest Magnetic Wireless Powerbank 5000Mah Battery Capacity for iPhone 16</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1084.2</v>
+        <v>942.96</v>
       </c>
       <c r="G30" t="n">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="H30" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>46237</v>
@@ -2494,7 +2494,7 @@
         <v>46270</v>
       </c>
       <c r="M30" t="n">
-        <v>24937</v>
+        <v>28289</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -2505,50 +2505,50 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5OF8HBIC</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>46244</v>
+        <v>46237</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>B0FSSCW7WZ</t>
+          <t>B0FT2VNW5H</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DUPLOBLK</t>
+          <t>WCZENO30WWHT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Stuffcool Duplo 140W Dual Type-C Cable 1.2m Nylon-Braided Dual USB-C Connectors with Smart E-Ma</t>
+          <t>Stuffcool Zeno 30W GaN Type C Fast Charger Retractable Cable 75cm PD PPS iPhone Pixel Samsung S</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>698.6900000000001</v>
+        <v>1084.2</v>
       </c>
       <c r="G31" t="n">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="H31" t="n">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="I31" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>46244</v>
+        <v>46237</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>46285</v>
+        <v>46266</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>46289</v>
+        <v>46270</v>
       </c>
       <c r="M31" t="n">
-        <v>24454</v>
+        <v>24937</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -2559,50 +2559,50 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>5OF8HBIC</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>46265</v>
+        <v>46244</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>B0FT2VNW5H</t>
+          <t>B0FSSCW7WZ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>WCZENO30WWHT</t>
+          <t>DUPLOBLK</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Stuffcool Zeno 30W GaN Type C Fast Charger Retractable Cable 75cm PD PPS iPhone Pixel Samsung S</t>
+          <t>Stuffcool Duplo 140W Dual Type-C Cable 1.2m Nylon-Braided Dual USB-C Connectors with Smart E-Ma</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1084.2</v>
+        <v>698.6900000000001</v>
       </c>
       <c r="G32" t="n">
-        <v>112</v>
+        <v>63</v>
       </c>
       <c r="H32" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="I32" t="n">
-        <v>91</v>
+        <v>28</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>46266</v>
+        <v>46244</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>46294</v>
+        <v>46285</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>46298</v>
+        <v>46289</v>
       </c>
       <c r="M32" t="n">
-        <v>22768</v>
+        <v>24454</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -2613,50 +2613,50 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>8Z6APQQC</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>46258</v>
+        <v>46265</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>B0H5HYK4KZ</t>
+          <t>B0FT2VNW5H</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>PBOMNIIVRY</t>
+          <t>WCZENO30WWHT</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Omni 3-in-1 10000mAh Magnetic Wireless Powerbank with Dedicated Apple Watch Charging </t>
+          <t>Stuffcool Zeno 30W GaN Type C Fast Charger Retractable Cable 75cm PD PPS iPhone Pixel Samsung S</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1692.59</v>
+        <v>1084.2</v>
       </c>
       <c r="G33" t="n">
-        <v>88</v>
+        <v>112</v>
       </c>
       <c r="H33" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="I33" t="n">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>46258</v>
+        <v>46266</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>46286</v>
+        <v>46294</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>46290</v>
+        <v>46298</v>
       </c>
       <c r="M33" t="n">
-        <v>20311</v>
+        <v>22768</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -2667,50 +2667,50 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>8Z6APQQC</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>46237</v>
+        <v>46258</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>B0H6J3YQ1D</t>
+          <t>B0H5HYK4KZ</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>WCNVS25CBLU</t>
+          <t>PBOMNIIVRY</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pixel &amp; iPhone Blue</t>
+          <t xml:space="preserve">Stuffcool Omni 3-in-1 10000mAh Magnetic Wireless Powerbank with Dedicated Apple Watch Charging </t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>433.36</v>
+        <v>1692.59</v>
       </c>
       <c r="G34" t="n">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="H34" t="n">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="I34" t="n">
-        <v>24</v>
+        <v>76</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>46237</v>
+        <v>46258</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>46266</v>
+        <v>46286</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="M34" t="n">
-        <v>19935</v>
+        <v>20311</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -2721,50 +2721,50 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5OF8HBIC</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>46244</v>
+        <v>46237</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>B0FV2VNK12</t>
+          <t>B0H6J3YQ1D</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>WCEMP75SIL</t>
+          <t>WCNVS25CBLU</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Stuffcool Empire 75W GaN Multiport Fast Charger with 4 Type-C &amp; 1 USB-A, Smart Power Distributi</t>
+          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pixel &amp; iPhone Blue</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2168.95</v>
+        <v>433.36</v>
       </c>
       <c r="G35" t="n">
-        <v>9</v>
+        <v>70</v>
       </c>
       <c r="H35" t="n">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>46244</v>
+        <v>46237</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>46285</v>
+        <v>46266</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>46289</v>
+        <v>46270</v>
       </c>
       <c r="M35" t="n">
-        <v>19521</v>
+        <v>19935</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -2775,50 +2775,50 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>53SMQFHQ</t>
+          <t>5OF8HBIC</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>46251</v>
+        <v>46244</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>B0FTFVKTH6</t>
+          <t>B0FV2VNK12</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ULTIMUS128BLK</t>
+          <t>WCEMP75SIL</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Stuffcool Ultimus 128W Super Fast Car Charger Dual Type-C USB-A PD 65W PD 30W QC 30W Compatible</t>
+          <t>Stuffcool Empire 75W GaN Multiport Fast Charger with 4 Type-C &amp; 1 USB-A, Smart Power Distributi</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1518.1</v>
+        <v>2168.95</v>
       </c>
       <c r="G36" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H36" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>46251</v>
+        <v>46244</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>46279</v>
+        <v>46285</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>46283</v>
+        <v>46289</v>
       </c>
       <c r="M36" t="n">
-        <v>16699</v>
+        <v>19521</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -2829,50 +2829,50 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>53SMQFHQ</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>46265</v>
+        <v>46251</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>B0FV2VNK12</t>
+          <t>B0FTFVKTH6</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>WCEMP75SIL</t>
+          <t>ULTIMUS128BLK</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Stuffcool Empire 75W GaN Multiport Fast Charger with 4 Type-C &amp; 1 USB-A, Smart Power Distributi</t>
+          <t>Stuffcool Ultimus 128W Super Fast Car Charger Dual Type-C USB-A PD 65W PD 30W QC 30W Compatible</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2168.95</v>
+        <v>1518.1</v>
       </c>
       <c r="G37" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="H37" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="I37" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>46266</v>
+        <v>46251</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>46294</v>
+        <v>46279</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>46298</v>
+        <v>46283</v>
       </c>
       <c r="M37" t="n">
-        <v>13014</v>
+        <v>16699</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -2883,50 +2883,50 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>46237</v>
+        <v>46265</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>B0DZHKBBM1</t>
+          <t>B0FV2VNK12</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>PBMAVERICKBLK</t>
+          <t>WCEMP75SIL</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Maverick Mini 20,000mAh Powerbank with 20W Built-in Lightning &amp; Type-C Cables, 22.5W </t>
+          <t>Stuffcool Empire 75W GaN Multiport Fast Charger with 4 Type-C &amp; 1 USB-A, Smart Power Distributi</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>1219.73</v>
+        <v>2168.95</v>
       </c>
       <c r="G38" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H38" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>46237</v>
+        <v>46266</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>46266</v>
+        <v>46294</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>46270</v>
+        <v>46298</v>
       </c>
       <c r="M38" t="n">
-        <v>12197</v>
+        <v>13014</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -2937,50 +2937,50 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>46265</v>
+        <v>46237</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>B0D3N594JW</t>
+          <t>B0DZHKBBM1</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>WRLREVELBLK</t>
+          <t>PBMAVERICKBLK</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Stuffcool Revel Magnetic Wireless Qi2 Certified Charger- Charges iPhone 12/13/14/15/16 and Andr</t>
+          <t xml:space="preserve">Stuffcool Maverick Mini 20,000mAh Powerbank with 20W Built-in Lightning &amp; Type-C Cables, 22.5W </t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>762.2</v>
+        <v>1219.73</v>
       </c>
       <c r="G39" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="H39" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="K39" s="3" t="n">
         <v>46266</v>
       </c>
-      <c r="K39" s="3" t="n">
-        <v>46294</v>
-      </c>
       <c r="L39" s="3" t="n">
-        <v>46298</v>
+        <v>46270</v>
       </c>
       <c r="M39" t="n">
-        <v>12195</v>
+        <v>12197</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -2991,50 +2991,50 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>8Z6APQQC</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>46258</v>
+        <v>46265</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>B0FTFVKTH6</t>
+          <t>B0D3N594JW</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ULTIMUS128BLK</t>
+          <t>WRLREVELBLK</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Stuffcool Ultimus 128W Super Fast Car Charger Dual Type-C USB-A PD 65W PD 30W QC 30W Compatible</t>
+          <t>Stuffcool Revel Magnetic Wireless Qi2 Certified Charger- Charges iPhone 12/13/14/15/16 and Andr</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>1518.1</v>
+        <v>762.2</v>
       </c>
       <c r="G40" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H40" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>46258</v>
+        <v>46266</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>46286</v>
+        <v>46294</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>46290</v>
+        <v>46298</v>
       </c>
       <c r="M40" t="n">
-        <v>12145</v>
+        <v>12195</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -3045,50 +3045,50 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>6WAHMIEG</t>
+          <t>8Z6APQQC</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>46252</v>
+        <v>46258</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>B0CCJ8BX6C</t>
+          <t>B0FTFVKTH6</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>PBCLICKGRY</t>
+          <t>ULTIMUS128BLK</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Stuffcool Click 5000mAh Made in India Magnetic Wireless Powerbank with 18W PD Fast Charing Type</t>
+          <t>Stuffcool Ultimus 128W Super Fast Car Charger Dual Type-C USB-A PD 65W PD 30W QC 30W Compatible</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>1185.85</v>
+        <v>1518.1</v>
       </c>
       <c r="G41" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H41" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I41" t="n">
         <v>0</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>46278</v>
+        <v>46258</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="M41" t="n">
-        <v>11858</v>
+        <v>12145</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -3099,50 +3099,50 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>8Z6APQQC</t>
+          <t>6WAHMIEG</t>
         </is>
       </c>
       <c r="B42" s="3" t="n">
-        <v>46258</v>
+        <v>46252</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>B0FV2VNK12</t>
+          <t>B0CCJ8BX6C</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>WCEMP75SIL</t>
+          <t>PBCLICKGRY</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Stuffcool Empire 75W GaN Multiport Fast Charger with 4 Type-C &amp; 1 USB-A, Smart Power Distributi</t>
+          <t>Stuffcool Click 5000mAh Made in India Magnetic Wireless Powerbank with 18W PD Fast Charing Type</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>2168.95</v>
+        <v>1185.85</v>
       </c>
       <c r="G42" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H42" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>46258</v>
+        <v>46278</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>46286</v>
+        <v>46285</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
       <c r="M42" t="n">
-        <v>10845</v>
+        <v>11858</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -3153,50 +3153,50 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>8Z6APQQC</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>46265</v>
+        <v>46258</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>B0BXXMZLDY</t>
+          <t>B0FV2VNK12</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>PBSP85WBLK</t>
+          <t>WCEMP75SIL</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Stuffcool Super Power 85W 20000mAh Powerbank Compatible to Charge Macbooks, Laptops, iPads, Tab</t>
+          <t>Stuffcool Empire 75W GaN Multiport Fast Charger with 4 Type-C &amp; 1 USB-A, Smart Power Distributi</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>2960.17</v>
+        <v>2168.95</v>
       </c>
       <c r="G43" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H43" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>46266</v>
+        <v>46258</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>46294</v>
+        <v>46286</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>46298</v>
+        <v>46290</v>
       </c>
       <c r="M43" t="n">
-        <v>5920</v>
+        <v>10845</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -3207,50 +3207,50 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>53SMQFHQ</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>46251</v>
+        <v>46265</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>B0H2VFTQ1C</t>
+          <t>B0BXXMZLDY</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>WCNUMEN45PROWHT</t>
+          <t>PBSP85WBLK</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Numen 45 Pro Dual Type-C GaN Charger with 45W PD PPS Fast Charging, Supports Samsung </t>
+          <t>Stuffcool Super Power 85W 20000mAh Powerbank Compatible to Charge Macbooks, Laptops, iPads, Tab</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>867.25</v>
+        <v>2960.17</v>
       </c>
       <c r="G44" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="H44" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I44" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>46251</v>
+        <v>46266</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>46279</v>
+        <v>46294</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>46283</v>
+        <v>46298</v>
       </c>
       <c r="M44" t="n">
-        <v>5204</v>
+        <v>5920</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
@@ -3261,50 +3261,50 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>53SMQFHQ</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>46237</v>
+        <v>46251</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>B0GZVCYSXL</t>
+          <t>B0H2VFTQ1C</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>WCNVS25CWHT</t>
+          <t>WCNUMEN45PROWHT</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pixel &amp; iPhone</t>
+          <t xml:space="preserve">Stuffcool Numen 45 Pro Dual Type-C GaN Charger with 45W PD PPS Fast Charging, Supports Samsung </t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>433.36</v>
+        <v>867.25</v>
       </c>
       <c r="G45" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H45" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>46237</v>
+        <v>46251</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>46266</v>
+        <v>46279</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>46270</v>
+        <v>46283</v>
       </c>
       <c r="M45" t="n">
-        <v>3467</v>
+        <v>5204</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -3315,50 +3315,50 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>5OF8HBIC</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>46244</v>
+        <v>46237</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>B0DFYZWRFQ</t>
+          <t>B0GZVCYSXL</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>PBROAM20WHT</t>
+          <t>WCNVS25CWHT</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Stuffcool Roam+ 20000mAh Compact Powerbank with 20W Type C Output Charges iPhone 50% in 30 mins</t>
+          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pixel &amp; iPhone</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1067.2</v>
+        <v>433.36</v>
       </c>
       <c r="G46" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="H46" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I46" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>46244</v>
+        <v>46237</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>46285</v>
+        <v>46266</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>46289</v>
+        <v>46270</v>
       </c>
       <c r="M46" t="n">
-        <v>3202</v>
+        <v>3467</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -3369,50 +3369,50 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>5OF8HBIC</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>46265</v>
+        <v>46244</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>B0DMVN35V5</t>
+          <t>B0DFYZWRFQ</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>RMSIP16PLBLK</t>
+          <t>PBROAM20WHT</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Stuffcool Rims Silicone case for iPhone 16 Plus, Magsafe Enabled with a Raised Metallic Frame f</t>
+          <t>Stuffcool Roam+ 20000mAh Compact Powerbank with 20W Type C Output Charges iPhone 50% in 30 mins</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>863.9</v>
+        <v>1067.2</v>
       </c>
       <c r="G47" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="H47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>46266</v>
+        <v>46244</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>46294</v>
+        <v>46285</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>46298</v>
+        <v>46289</v>
       </c>
       <c r="M47" t="n">
-        <v>1728</v>
+        <v>3202</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
@@ -3423,50 +3423,50 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>8Z6APQQC</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="B48" s="3" t="n">
-        <v>46258</v>
+        <v>46265</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>B0DB1MXGD4</t>
+          <t>B0DMVN35V5</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>PBCLICKMAXWHT</t>
+          <t>RMSIP16PLBLK</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Click Max 10000mAh Powerbank with Built-in PD20W Type-C Cable to Fast Charge iPhones </t>
+          <t>Stuffcool Rims Silicone case for iPhone 16 Plus, Magsafe Enabled with a Raised Metallic Frame f</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1363.81</v>
+        <v>863.9</v>
       </c>
       <c r="G48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>46258</v>
+        <v>46266</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>46286</v>
+        <v>46294</v>
       </c>
       <c r="L48" s="3" t="n">
-        <v>46290</v>
+        <v>46298</v>
       </c>
       <c r="M48" t="n">
-        <v>1364</v>
+        <v>1728</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
@@ -3477,29 +3477,29 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>8Z6APQQC</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>46237</v>
+        <v>46258</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>B0DDTL6R6Y</t>
+          <t>B0DB1MXGD4</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>PBMEGAII30WGRN</t>
+          <t>PBCLICKMAXWHT</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Stuffcool Mega II Compact 10,000mAh 25W Powerbank with Samsung Super Fast Charging, Charges iPh</t>
+          <t xml:space="preserve">Stuffcool Click Max 10000mAh Powerbank with Built-in PD20W Type-C Cable to Fast Charge iPhones </t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>889.24</v>
+        <v>1363.81</v>
       </c>
       <c r="G49" t="n">
         <v>1</v>
@@ -3511,16 +3511,16 @@
         <v>0</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>46237</v>
+        <v>46258</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>46266</v>
+        <v>46286</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="M49" t="n">
-        <v>889</v>
+        <v>1364</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
@@ -3531,50 +3531,50 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>5OF8HBIC</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
-        <v>46244</v>
+        <v>46237</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>B0GZVCYSXL</t>
+          <t>B0DDTL6R6Y</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>WCNVS25CWHT</t>
+          <t>PBMEGAII30WGRN</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pixel &amp; iPhone</t>
+          <t>Stuffcool Mega II Compact 10,000mAh 25W Powerbank with Samsung Super Fast Charging, Charges iPh</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>433.36</v>
+        <v>889.24</v>
       </c>
       <c r="G50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>46244</v>
+        <v>46237</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>46285</v>
+        <v>46266</v>
       </c>
       <c r="L50" s="3" t="n">
-        <v>46289</v>
+        <v>46270</v>
       </c>
       <c r="M50" t="n">
-        <v>867</v>
+        <v>889</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -3585,59 +3585,113 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>5OF8HBIC</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>B0GZVCYSXL</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>WCNVS25CWHT</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pixel &amp; iPhone</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>433.36</v>
+      </c>
+      <c r="G51" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" t="n">
+        <v>2</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="3" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K51" s="3" t="n">
+        <v>46285</v>
+      </c>
+      <c r="L51" s="3" t="n">
+        <v>46289</v>
+      </c>
+      <c r="M51" t="n">
+        <v>867</v>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>P1-Incumbent (running down)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>39VRVKCF</t>
         </is>
       </c>
-      <c r="B51" s="3" t="n">
+      <c r="B52" s="3" t="n">
         <v>46237</v>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>B0C7QBPS1H</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>QUADN1BLK</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t xml:space="preserve">Stuffcool Quad 4 in 1 Cable 65W PD USB to Lightning, USB to Type-C, Type-C to Lightning &amp; Type </t>
         </is>
       </c>
-      <c r="F51" t="n">
+      <c r="F52" t="n">
         <v>296.19</v>
       </c>
-      <c r="G51" t="n">
+      <c r="G52" t="n">
         <v>1</v>
       </c>
-      <c r="H51" t="n">
+      <c r="H52" t="n">
         <v>1</v>
       </c>
-      <c r="I51" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" s="3" t="n">
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="3" t="n">
         <v>46237</v>
       </c>
-      <c r="K51" s="3" t="n">
+      <c r="K52" s="3" t="n">
         <v>46266</v>
       </c>
-      <c r="L51" s="3" t="n">
+      <c r="L52" s="3" t="n">
         <v>46270</v>
       </c>
-      <c r="M51" t="n">
+      <c r="M52" t="n">
         <v>296</v>
       </c>
-      <c r="N51" t="inlineStr">
+      <c r="N52" t="inlineStr">
         <is>
           <t>P1-Incumbent (running down)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N51"/>
+  <autoFilter ref="A1:N52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5271,17 +5325,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>B0FTFVKTH6</t>
+          <t>B0D8443PTW</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ULTIMUS128BLK</t>
+          <t>QUADPROMAXBLK</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Ultimus 128W Super Fast Car Charger Dual Type-C </t>
+          <t>Stuffcool Quad Pro Max 4 in 1 Metal Braided Cable 1.5m 240</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -5290,41 +5344,41 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>33</v>
+        <v>360</v>
       </c>
       <c r="H25" t="n">
-        <v>1.666666666666667</v>
+        <v>12</v>
       </c>
       <c r="I25" t="n">
-        <v>19.8</v>
+        <v>30</v>
       </c>
       <c r="J25" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="K25" t="n">
-        <v>19</v>
+        <v>72</v>
       </c>
       <c r="L25" t="n">
-        <v>19</v>
+        <v>60</v>
       </c>
       <c r="M25" t="n">
-        <v>31.2</v>
+        <v>35</v>
       </c>
       <c r="N25" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="O25" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>1518.1</v>
+        <v>508.05</v>
       </c>
       <c r="Q25" t="n">
-        <v>28844</v>
+        <v>30483</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>53SMQFHQ, 8Z6APQQC</t>
+          <t>5OF8HBIC</t>
         </is>
       </c>
       <c r="S25" t="b">
@@ -5334,17 +5388,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>B0DPHR4FG7</t>
+          <t>B0FTFVKTH6</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PBLUCIDWHT</t>
+          <t>ULTIMUS128BLK</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Stuffcool Lucid 15W Smallest Magnetic Wireless Powerbank 5</t>
+          <t xml:space="preserve">Stuffcool Ultimus 128W Super Fast Car Charger Dual Type-C </t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5353,40 +5407,41 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>1.666666666666667</v>
+      </c>
+      <c r="I26" t="n">
+        <v>19.8</v>
       </c>
       <c r="J26" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="K26" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="L26" t="n">
-        <v>30</v>
+        <v>19</v>
+      </c>
+      <c r="M26" t="n">
+        <v>31.2</v>
       </c>
       <c r="N26" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P26" t="n">
-        <v>942.96</v>
+        <v>1518.1</v>
       </c>
       <c r="Q26" t="n">
-        <v>28289</v>
+        <v>28844</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>53SMQFHQ, 8Z6APQQC</t>
         </is>
       </c>
       <c r="S26" t="b">
@@ -5396,17 +5451,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>B0FSSCW7WZ</t>
+          <t>B0DPHR4FG7</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DUPLOBLK</t>
+          <t>PBLUCIDWHT</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Duplo 140W Dual Type-C Cable 1.2m Nylon-Braided </t>
+          <t>Stuffcool Lucid 15W Smallest Magnetic Wireless Powerbank 5</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -5415,41 +5470,40 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>1.333333333333333</v>
-      </c>
-      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>30</v>
+      </c>
+      <c r="K27" t="n">
+        <v>39</v>
+      </c>
+      <c r="L27" t="n">
+        <v>30</v>
+      </c>
+      <c r="N27" t="n">
         <v>9</v>
       </c>
-      <c r="J27" t="n">
-        <v>35</v>
-      </c>
-      <c r="K27" t="n">
-        <v>79</v>
-      </c>
-      <c r="L27" t="n">
-        <v>35</v>
-      </c>
-      <c r="M27" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="N27" t="n">
-        <v>44</v>
-      </c>
       <c r="O27" t="n">
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>698.6900000000001</v>
+        <v>942.96</v>
       </c>
       <c r="Q27" t="n">
-        <v>24454</v>
+        <v>28289</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>53SMQFHQ, 5OF8HBIC</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="S27" t="b">
@@ -5459,17 +5513,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>B0H5HYK4KZ</t>
+          <t>B0FSSCW7WZ</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PBOMNIIVRY</t>
+          <t>DUPLOBLK</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Stuffcool Omni 3-in-1 10000mAh Magnetic Wireless Powerbank</t>
+          <t xml:space="preserve">Stuffcool Duplo 140W Dual Type-C Cable 1.2m Nylon-Braided </t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -5478,41 +5532,41 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="H28" t="n">
-        <v>2.666666666666667</v>
+        <v>1.333333333333333</v>
       </c>
       <c r="I28" t="n">
-        <v>30.375</v>
+        <v>9</v>
       </c>
       <c r="J28" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="K28" t="n">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="L28" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="M28" t="n">
-        <v>34.9</v>
+        <v>35.2</v>
       </c>
       <c r="N28" t="n">
-        <v>85</v>
+        <v>44</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>1692.59</v>
+        <v>698.6900000000001</v>
       </c>
       <c r="Q28" t="n">
-        <v>20311</v>
+        <v>24454</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>5FPANY5G, 8Z6APQQC</t>
+          <t>53SMQFHQ, 5OF8HBIC</t>
         </is>
       </c>
       <c r="S28" t="b">
@@ -5522,17 +5576,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>B0H6J3YQ1D</t>
+          <t>B0H5HYK4KZ</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>WCNVS25CBLU</t>
+          <t>PBOMNIIVRY</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pi</t>
+          <t>Stuffcool Omni 3-in-1 10000mAh Magnetic Wireless Powerbank</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -5541,41 +5595,41 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="H29" t="n">
-        <v>2</v>
+        <v>2.666666666666667</v>
       </c>
       <c r="I29" t="n">
+        <v>30.375</v>
+      </c>
+      <c r="J29" t="n">
         <v>12</v>
       </c>
-      <c r="J29" t="n">
-        <v>46</v>
-      </c>
       <c r="K29" t="n">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="L29" t="n">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="M29" t="n">
-        <v>35</v>
+        <v>34.9</v>
       </c>
       <c r="N29" t="n">
-        <v>43</v>
+        <v>85</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>433.36</v>
+        <v>1692.59</v>
       </c>
       <c r="Q29" t="n">
-        <v>19935</v>
+        <v>20311</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>39VRVKCF, 53SMQFHQ, 8Z6APQQC</t>
+          <t>5FPANY5G, 8Z6APQQC</t>
         </is>
       </c>
       <c r="S29" t="b">
@@ -5585,17 +5639,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>B0D3N594JW</t>
+          <t>B0H6J3YQ1D</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>WRLREVELBLK</t>
+          <t>WCNVS25CBLU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Stuffcool Revel Magnetic Wireless Qi2 Certified Charger- C</t>
+          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pi</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -5604,40 +5658,41 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="I30" t="n">
+        <v>12</v>
       </c>
       <c r="J30" t="n">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="K30" t="n">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="L30" t="n">
-        <v>16</v>
+        <v>46</v>
+      </c>
+      <c r="M30" t="n">
+        <v>35</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>762.2</v>
+        <v>433.36</v>
       </c>
       <c r="Q30" t="n">
-        <v>12195</v>
+        <v>19935</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>39VRVKCF, 53SMQFHQ, 8Z6APQQC</t>
         </is>
       </c>
       <c r="S30" t="b">
@@ -5647,17 +5702,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>B0CCJ8BX6C</t>
+          <t>B0D3N594JW</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PBCLICKGRY</t>
+          <t>WRLREVELBLK</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Stuffcool Click 5000mAh Made in India Magnetic Wireless Po</t>
+          <t>Stuffcool Revel Magnetic Wireless Qi2 Certified Charger- C</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -5677,13 +5732,13 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="K31" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="L31" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="N31" t="n">
         <v>0</v>
@@ -5692,14 +5747,14 @@
         <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>1185.85</v>
+        <v>762.2</v>
       </c>
       <c r="Q31" t="n">
-        <v>11858</v>
+        <v>12195</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>6WAHMIEG</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="S31" t="b">
@@ -5709,17 +5764,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>B0BXXMZLDY</t>
+          <t>B0CCJ8BX6C</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PBSP85WBLK</t>
+          <t>PBCLICKGRY</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Stuffcool Super Power 85W 20000mAh Powerbank Compatible to</t>
+          <t>Stuffcool Click 5000mAh Made in India Magnetic Wireless Po</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -5739,13 +5794,13 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K32" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L32" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="N32" t="n">
         <v>0</v>
@@ -5754,14 +5809,14 @@
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>2960.17</v>
+        <v>1185.85</v>
       </c>
       <c r="Q32" t="n">
-        <v>5920</v>
+        <v>11858</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>6WAHMIEG</t>
         </is>
       </c>
       <c r="S32" t="b">
@@ -5771,17 +5826,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>B0H2VFTQ1C</t>
+          <t>B0BXXMZLDY</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>WCNUMEN45PROWHT</t>
+          <t>PBSP85WBLK</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Stuffcool Numen 45 Pro Dual Type-C GaN Charger with 45W PD</t>
+          <t>Stuffcool Super Power 85W 20000mAh Powerbank Compatible to</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -5790,41 +5845,40 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>5</v>
-      </c>
-      <c r="I33" t="n">
-        <v>33.8</v>
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="J33" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K33" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="L33" t="n">
-        <v>6</v>
-      </c>
-      <c r="M33" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="N33" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>867.25</v>
+        <v>2960.17</v>
       </c>
       <c r="Q33" t="n">
-        <v>5204</v>
+        <v>5920</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>53SMQFHQ, 8Z6APQQC</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="S33" t="b">
@@ -5834,17 +5888,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>B0GZVCYSXL</t>
+          <t>B0H2VFTQ1C</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>WCNVS25CWHT</t>
+          <t>WCNUMEN45PROWHT</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pi</t>
+          <t>Stuffcool Numen 45 Pro Dual Type-C GaN Charger with 45W PD</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -5853,41 +5907,41 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>58</v>
+        <v>169</v>
       </c>
       <c r="H34" t="n">
-        <v>3.666666666666667</v>
+        <v>5</v>
       </c>
       <c r="I34" t="n">
-        <v>15.81818181818182</v>
+        <v>33.8</v>
       </c>
       <c r="J34" t="n">
-        <v>70</v>
+        <v>6</v>
       </c>
       <c r="K34" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="L34" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="M34" t="n">
-        <v>18.5</v>
+        <v>35</v>
       </c>
       <c r="N34" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="O34" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>433.36</v>
+        <v>867.25</v>
       </c>
       <c r="Q34" t="n">
-        <v>4334</v>
+        <v>5204</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>39VRVKCF, 5OF8HBIC</t>
+          <t>53SMQFHQ, 8Z6APQQC</t>
         </is>
       </c>
       <c r="S34" t="b">
@@ -5897,17 +5951,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>B0DFYZWRFQ</t>
+          <t>B0GZVCYSXL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PBROAM20WHT</t>
+          <t>WCNVS25CWHT</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Stuffcool Roam+ 20000mAh Compact Powerbank with 20W Type C</t>
+          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pi</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -5916,41 +5970,41 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="H35" t="n">
-        <v>0.3333333333333333</v>
+        <v>3.666666666666667</v>
       </c>
       <c r="I35" t="n">
-        <v>27</v>
+        <v>15.81818181818182</v>
       </c>
       <c r="J35" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="K35" t="n">
-        <v>217</v>
+        <v>10</v>
       </c>
       <c r="L35" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="M35" t="n">
-        <v>36</v>
+        <v>18.5</v>
       </c>
       <c r="N35" t="n">
-        <v>214</v>
+        <v>0</v>
       </c>
       <c r="O35" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="P35" t="n">
-        <v>1067.2</v>
+        <v>433.36</v>
       </c>
       <c r="Q35" t="n">
-        <v>3202</v>
+        <v>4334</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>53SMQFHQ, 5OF8HBIC, 8Z6APQQC</t>
+          <t>39VRVKCF, 5OF8HBIC</t>
         </is>
       </c>
       <c r="S35" t="b">
@@ -5960,17 +6014,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>B0DMVN35V5</t>
+          <t>B0DFYZWRFQ</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>RMSIP16PLBLK</t>
+          <t>PBROAM20WHT</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Stuffcool Rims Silicone case for iPhone 16 Plus, Magsafe E</t>
+          <t>Stuffcool Roam+ 20000mAh Compact Powerbank with 20W Type C</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -5979,40 +6033,41 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="I36" t="n">
+        <v>27</v>
       </c>
       <c r="J36" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="K36" t="n">
-        <v>2</v>
+        <v>217</v>
       </c>
       <c r="L36" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="M36" t="n">
+        <v>36</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>214</v>
       </c>
       <c r="O36" t="n">
         <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>863.9</v>
+        <v>1067.2</v>
       </c>
       <c r="Q36" t="n">
-        <v>1728</v>
+        <v>3202</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>53SMQFHQ, 5OF8HBIC, 8Z6APQQC</t>
         </is>
       </c>
       <c r="S36" t="b">
@@ -6022,17 +6077,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>B0DB1MXGD4</t>
+          <t>B0DMVN35V5</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PBCLICKMAXWHT</t>
+          <t>RMSIP16PLBLK</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Stuffcool Click Max 10000mAh Powerbank with Built-in PD20W</t>
+          <t>Stuffcool Rims Silicone case for iPhone 16 Plus, Magsafe E</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -6052,13 +6107,13 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N37" t="n">
         <v>0</v>
@@ -6067,14 +6122,14 @@
         <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>1363.81</v>
+        <v>863.9</v>
       </c>
       <c r="Q37" t="n">
-        <v>1364</v>
+        <v>1728</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>8Z6APQQC</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="S37" t="b">
@@ -6084,17 +6139,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>B0DDTL6R6Y</t>
+          <t>B0DB1MXGD4</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PBMEGAII30WGRN</t>
+          <t>PBCLICKMAXWHT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Stuffcool Mega II Compact 10,000mAh 25W Powerbank with Sam</t>
+          <t>Stuffcool Click Max 10000mAh Powerbank with Built-in PD20W</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -6129,14 +6184,14 @@
         <v>0</v>
       </c>
       <c r="P38" t="n">
-        <v>889.24</v>
+        <v>1363.81</v>
       </c>
       <c r="Q38" t="n">
-        <v>889</v>
+        <v>1364</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>8Z6APQQC</t>
         </is>
       </c>
       <c r="S38" t="b">
@@ -6146,17 +6201,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>B0C7QBPS1H</t>
+          <t>B0DDTL6R6Y</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>QUADN1BLK</t>
+          <t>PBMEGAII30WGRN</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Stuffcool Quad 4 in 1 Cable 65W PD USB to Lightning, USB t</t>
+          <t>Stuffcool Mega II Compact 10,000mAh 25W Powerbank with Sam</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -6191,10 +6246,10 @@
         <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v>296.19</v>
+        <v>889.24</v>
       </c>
       <c r="Q39" t="n">
-        <v>296</v>
+        <v>889</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
@@ -6208,17 +6263,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>B0C3GT42X5</t>
+          <t>B0C7QBPS1H</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>WCNOVA65WWHT</t>
+          <t>QUADN1BLK</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Stuffcool Nova 65W Gan Charger Made in India 3 Ports Suppo</t>
+          <t>Stuffcool Quad 4 in 1 Cable 65W PD USB to Lightning, USB t</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -6227,7 +6282,7 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -6238,13 +6293,13 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N40" t="n">
         <v>0</v>
@@ -6253,10 +6308,15 @@
         <v>0</v>
       </c>
       <c r="P40" t="n">
-        <v>1270.68</v>
+        <v>296.19</v>
       </c>
       <c r="Q40" t="n">
-        <v>0</v>
+        <v>296</v>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>39VRVKCF</t>
+        </is>
       </c>
       <c r="S40" t="b">
         <v>0</v>
@@ -6265,17 +6325,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>B0CMTDGZSP</t>
+          <t>B0C3GT42X5</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>WCNV20WHT</t>
+          <t>WCNOVA65WWHT</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Nuevo PD20W Made in India Smallest Wall Charger </t>
+          <t>Stuffcool Nova 65W Gan Charger Made in India 3 Ports Suppo</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -6284,7 +6344,7 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -6310,7 +6370,7 @@
         <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>304.58</v>
+        <v>1270.68</v>
       </c>
       <c r="Q41" t="n">
         <v>0</v>
@@ -6322,17 +6382,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>B0D8443PTW</t>
+          <t>B0CMTDGZSP</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>QUADPROMAXBLK</t>
+          <t>WCNV20WHT</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Stuffcool Quad Pro Max 4 in 1 Metal Braided Cable 1.5m 240</t>
+          <t xml:space="preserve">Stuffcool Nuevo PD20W Made in India Smallest Wall Charger </t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -6340,48 +6400,37 @@
           <t>P1-Incumbent (running down)</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Quad Pro cable</t>
-        </is>
-      </c>
       <c r="G42" t="n">
-        <v>360</v>
+        <v>3</v>
       </c>
       <c r="H42" t="n">
-        <v>12</v>
-      </c>
-      <c r="I42" t="n">
-        <v>30</v>
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="J42" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
         <v>0</v>
       </c>
-      <c r="M42" t="n">
-        <v>30</v>
-      </c>
       <c r="N42" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="O42" t="n">
         <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>508.05</v>
+        <v>304.58</v>
       </c>
       <c r="Q42" t="n">
         <v>0</v>
-      </c>
-      <c r="R42" t="inlineStr">
-        <is>
-          <t>5OF8HBIC</t>
-        </is>
       </c>
       <c r="S42" t="b">
         <v>0</v>
@@ -9739,7 +9788,7 @@
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
@@ -9826,7 +9875,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Quad Pro cable</t>
+          <t>Quad Pro cables (coexist)</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -9836,13 +9885,13 @@
         <v>360</v>
       </c>
       <c r="D4" t="n">
-        <v>300</v>
+        <v>360</v>
       </c>
       <c r="E4" t="n">
-        <v>660</v>
+        <v>720</v>
       </c>
       <c r="F4" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -11571,44 +11620,44 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>5OF8HBIC</t>
+          <t>53SMQFHQ</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>B0D8443PTW</t>
+          <t>B0DFYZWRFQ</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>QUADPROMAXBLK</t>
+          <t>PBROAM20WHT</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Stuffcool Quad Pro Max 4 in 1 Metal Braided Cable 1.5m 240W Rugged e-Marker chip gold plated co</t>
+          <t>Stuffcool Roam+ 20000mAh Compact Powerbank with 20W Type C Output Charges iPhone 50% in 30 mins</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="J29" t="n">
-        <v>508.05</v>
+        <v>1067.2</v>
       </c>
       <c r="K29" t="n">
-        <v>36580</v>
+        <v>33083</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>46289</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="30">
@@ -11619,44 +11668,44 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>53SMQFHQ</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>46251</v>
+        <v>46265</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>B0DFYZWRFQ</t>
+          <t>B0FV2VNK12</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PBROAM20WHT</t>
+          <t>WCEMP75SIL</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Stuffcool Roam+ 20000mAh Compact Powerbank with 20W Type C Output Charges iPhone 50% in 30 mins</t>
+          <t>Stuffcool Empire 75W GaN Multiport Fast Charger with 4 Type-C &amp; 1 USB-A, Smart Power Distributi</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I30" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="J30" t="n">
-        <v>1067.2</v>
+        <v>2168.95</v>
       </c>
       <c r="K30" t="n">
-        <v>33083</v>
+        <v>30365</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>46283</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="31">
@@ -11667,44 +11716,44 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>5OF8HBIC</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>46265</v>
+        <v>46244</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>B0FV2VNK12</t>
+          <t>B0DFYZWRFQ</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>WCEMP75SIL</t>
+          <t>PBROAM20WHT</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Stuffcool Empire 75W GaN Multiport Fast Charger with 4 Type-C &amp; 1 USB-A, Smart Power Distributi</t>
+          <t>Stuffcool Roam+ 20000mAh Compact Powerbank with 20W Type C Output Charges iPhone 50% in 30 mins</t>
         </is>
       </c>
       <c r="G31" t="n">
+        <v>23</v>
+      </c>
+      <c r="H31" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" t="n">
         <v>20</v>
       </c>
-      <c r="H31" t="n">
-        <v>6</v>
-      </c>
-      <c r="I31" t="n">
-        <v>14</v>
-      </c>
       <c r="J31" t="n">
-        <v>2168.95</v>
+        <v>1067.2</v>
       </c>
       <c r="K31" t="n">
-        <v>30365</v>
+        <v>21344</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>46298</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="32">
@@ -11723,33 +11772,33 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>B0DFYZWRFQ</t>
+          <t>B0FSSCW7WZ</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PBROAM20WHT</t>
+          <t>DUPLOBLK</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Stuffcool Roam+ 20000mAh Compact Powerbank with 20W Type C Output Charges iPhone 50% in 30 mins</t>
+          <t>Stuffcool Duplo 140W Dual Type-C Cable 1.2m Nylon-Braided Dual USB-C Connectors with Smart E-Ma</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="H32" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="I32" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="J32" t="n">
-        <v>1067.2</v>
+        <v>698.6900000000001</v>
       </c>
       <c r="K32" t="n">
-        <v>21344</v>
+        <v>19563</v>
       </c>
       <c r="L32" s="3" t="n">
         <v>46289</v>
@@ -11763,44 +11812,44 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>5OF8HBIC</t>
+          <t>53SMQFHQ</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>B0FSSCW7WZ</t>
+          <t>B0H6J36G1L</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>DUPLOBLK</t>
+          <t>HKNVS25CCWHT</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Stuffcool Duplo 140W Dual Type-C Cable 1.2m Nylon-Braided Dual USB-C Connectors with Smart E-Ma</t>
+          <t>Stuffcool Novus 25W Super Fast GaN Charger with Type C to C 60W 3A Cable for Samsung, Pixel &amp; i</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="H33" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
         <v>28</v>
       </c>
       <c r="J33" t="n">
-        <v>698.6900000000001</v>
+        <v>650.3099999999999</v>
       </c>
       <c r="K33" t="n">
-        <v>19563</v>
+        <v>18209</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>46289</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="34">
@@ -11811,44 +11860,44 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>53SMQFHQ</t>
+          <t>8Z6APQQC</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>46251</v>
+        <v>46258</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>B0H6J36G1L</t>
+          <t>B0H6Q2YQ9C</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>HKNVS25CCWHT</t>
+          <t>PBOMNIPROSIL</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Stuffcool Novus 25W Super Fast GaN Charger with Type C to C 60W 3A Cable for Samsung, Pixel &amp; i</t>
+          <t>Stuffcool Omni Pro Qi2.2 Certified 25W MagSafe Powerbank 10000mAh with Apple Watch Charger, 35W</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I34" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="J34" t="n">
-        <v>650.3099999999999</v>
+        <v>3134.97</v>
       </c>
       <c r="K34" t="n">
-        <v>18209</v>
+        <v>15675</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>46283</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="35">
@@ -11859,44 +11908,44 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>8Z6APQQC</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>46258</v>
+        <v>46265</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>B0H6Q2YQ9C</t>
+          <t>B0H5HYK4KZ</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>PBOMNIPROSIL</t>
+          <t>PBOMNIIVRY</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Stuffcool Omni Pro Qi2.2 Certified 25W MagSafe Powerbank 10000mAh with Apple Watch Charger, 35W</t>
+          <t xml:space="preserve">Stuffcool Omni 3-in-1 10000mAh Magnetic Wireless Powerbank with Dedicated Apple Watch Charging </t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="H35" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="J35" t="n">
-        <v>3134.97</v>
+        <v>1692.59</v>
       </c>
       <c r="K35" t="n">
-        <v>15675</v>
+        <v>15233</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>46290</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="36">
@@ -11907,44 +11956,44 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>53SMQFHQ</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>46265</v>
+        <v>46251</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>B0H5HYK4KZ</t>
+          <t>B0H552PBFY</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>PBOMNIIVRY</t>
+          <t>HKNVS25CCORG</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Omni 3-in-1 10000mAh Magnetic Wireless Powerbank with Dedicated Apple Watch Charging </t>
+          <t>Stuffcool Novus 25W Super Fast GaN Charger with Type C to C 60W 3A Cable for Samsung, Pixel &amp; i</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="J36" t="n">
-        <v>1692.59</v>
+        <v>650.3099999999999</v>
       </c>
       <c r="K36" t="n">
-        <v>15233</v>
+        <v>13006</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>46298</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="37">
@@ -11963,33 +12012,33 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>B0H552PBFY</t>
+          <t>B0FSSCW7WZ</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>HKNVS25CCORG</t>
+          <t>DUPLOBLK</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Stuffcool Novus 25W Super Fast GaN Charger with Type C to C 60W 3A Cable for Samsung, Pixel &amp; i</t>
+          <t>Stuffcool Duplo 140W Dual Type-C Cable 1.2m Nylon-Braided Dual USB-C Connectors with Smart E-Ma</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J37" t="n">
-        <v>650.3099999999999</v>
+        <v>698.6900000000001</v>
       </c>
       <c r="K37" t="n">
-        <v>13006</v>
+        <v>11179</v>
       </c>
       <c r="L37" s="3" t="n">
         <v>46283</v>
@@ -12003,44 +12052,44 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>53SMQFHQ</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>46251</v>
+        <v>46265</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>B0FSSCW7WZ</t>
+          <t>B0GN99CJ8F</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>DUPLOBLK</t>
+          <t>WCZENO100WWHT</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Stuffcool Duplo 140W Dual Type-C Cable 1.2m Nylon-Braided Dual USB-C Connectors with Smart E-Ma</t>
+          <t xml:space="preserve">Stuffcool Zeno 100W Desktop Charging Station, 65W Retractable Type-C Cable, Dual 100W PD 3.0 &amp; </t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="J38" t="n">
-        <v>698.6900000000001</v>
+        <v>2168.95</v>
       </c>
       <c r="K38" t="n">
-        <v>11179</v>
+        <v>10845</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>46283</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="39">
@@ -12051,44 +12100,44 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>46265</v>
+        <v>46237</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>B0GN99CJ8F</t>
+          <t>B0H6J3YQ1D</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>WCZENO100WWHT</t>
+          <t>WCNVS25CBLU</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Zeno 100W Desktop Charging Station, 65W Retractable Type-C Cable, Dual 100W PD 3.0 &amp; </t>
+          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pixel &amp; iPhone Blue</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>5</v>
+        <v>70</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="I39" t="n">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="J39" t="n">
-        <v>2168.95</v>
+        <v>433.36</v>
       </c>
       <c r="K39" t="n">
-        <v>10845</v>
+        <v>10401</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>46298</v>
+        <v>46270</v>
       </c>
     </row>
     <row r="40">
@@ -12099,44 +12148,44 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>53SMQFHQ</t>
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>46237</v>
+        <v>46251</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>B0H6J3YQ1D</t>
+          <t>B0H2VFTQ1C</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>WCNVS25CBLU</t>
+          <t>WCNUMEN45PROWHT</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Stuffcool Novus 25W Super Fast GaN Charger for Samsung, Pixel &amp; iPhone Blue</t>
+          <t xml:space="preserve">Stuffcool Numen 45 Pro Dual Type-C GaN Charger with 45W PD PPS Fast Charging, Supports Samsung </t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>70</v>
+        <v>16</v>
       </c>
       <c r="H40" t="n">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="I40" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="J40" t="n">
-        <v>433.36</v>
+        <v>867.25</v>
       </c>
       <c r="K40" t="n">
-        <v>10401</v>
+        <v>8672</v>
       </c>
       <c r="L40" s="3" t="n">
-        <v>46270</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="41">
@@ -12147,44 +12196,44 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>53SMQFHQ</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>46251</v>
+        <v>46237</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>B0H2VFTQ1C</t>
+          <t>B0DPHR4FG7</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>WCNUMEN45PROWHT</t>
+          <t>PBLUCIDWHT</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stuffcool Numen 45 Pro Dual Type-C GaN Charger with 45W PD PPS Fast Charging, Supports Samsung </t>
+          <t>Stuffcool Lucid 15W Smallest Magnetic Wireless Powerbank 5000Mah Battery Capacity for iPhone 16</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="H41" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="I41" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J41" t="n">
-        <v>867.25</v>
+        <v>942.96</v>
       </c>
       <c r="K41" t="n">
-        <v>8672</v>
+        <v>8487</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>46283</v>
+        <v>46270</v>
       </c>
     </row>
     <row r="42">
@@ -12195,44 +12244,44 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>5OF8HBIC</t>
         </is>
       </c>
       <c r="C42" s="3" t="n">
-        <v>46237</v>
+        <v>46244</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>B0DPHR4FG7</t>
+          <t>B0GZBJRKSM</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>PBLUCIDWHT</t>
+          <t>PRIMUS1BLK</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Stuffcool Lucid 15W Smallest Magnetic Wireless Powerbank 5000Mah Battery Capacity for iPhone 16</t>
+          <t>Stuffcool Primus USB 4 Type-C to Type-C Cable with 240W Power and 40Gbps Data with 8K Video Tra</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="H42" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="J42" t="n">
-        <v>942.96</v>
+        <v>605.3</v>
       </c>
       <c r="K42" t="n">
-        <v>8487</v>
+        <v>8474</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>46270</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="43">
@@ -12243,11 +12292,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>5OF8HBIC</t>
+          <t>8Z6APQQC</t>
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>46244</v>
+        <v>46258</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -12265,22 +12314,22 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
       </c>
       <c r="I43" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J43" t="n">
         <v>605.3</v>
       </c>
       <c r="K43" t="n">
-        <v>8474</v>
+        <v>7264</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="44">
@@ -12291,44 +12340,44 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>8Z6APQQC</t>
+          <t>5OF8HBIC</t>
         </is>
       </c>
       <c r="C44" s="3" t="n">
-        <v>46258</v>
+        <v>46244</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>B0GZBJRKSM</t>
+          <t>B0H552PBFY</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>PRIMUS1BLK</t>
+          <t>HKNVS25CCORG</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Stuffcool Primus USB 4 Type-C to Type-C Cable with 240W Power and 40Gbps Data with 8K Video Tra</t>
+          <t>Stuffcool Novus 25W Super Fast GaN Charger with Type C to C 60W 3A Cable for Samsung, Pixel &amp; i</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J44" t="n">
-        <v>605.3</v>
+        <v>650.3099999999999</v>
       </c>
       <c r="K44" t="n">
-        <v>7264</v>
+        <v>6503</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>46290</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="45">
@@ -12395,33 +12444,33 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>B0H552PBFY</t>
+          <t>B0D8443PTW</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>HKNVS25CCORG</t>
+          <t>QUADPROMAXBLK</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Stuffcool Novus 25W Super Fast GaN Charger with Type C to C 60W 3A Cable for Samsung, Pixel &amp; i</t>
+          <t>Stuffcool Quad Pro Max 4 in 1 Metal Braided Cable 1.5m 240W Rugged e-Marker chip gold plated co</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>10</v>
+        <v>72</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="I46" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J46" t="n">
-        <v>650.3099999999999</v>
+        <v>508.05</v>
       </c>
       <c r="K46" t="n">
-        <v>6503</v>
+        <v>6097</v>
       </c>
       <c r="L46" s="3" t="n">
         <v>46289</v>
@@ -12867,11 +12916,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>53SMQFHQ</t>
         </is>
       </c>
       <c r="C56" s="3" t="n">
-        <v>46237</v>
+        <v>46251</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -12904,7 +12953,7 @@
         <v>2076</v>
       </c>
       <c r="L56" s="3" t="n">
-        <v>46270</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="57">
@@ -12915,11 +12964,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>53SMQFHQ</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="C57" s="3" t="n">
-        <v>46251</v>
+        <v>46237</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -12952,7 +13001,7 @@
         <v>2076</v>
       </c>
       <c r="L57" s="3" t="n">
-        <v>46283</v>
+        <v>46270</v>
       </c>
     </row>
     <row r="58">
@@ -13011,20 +13060,20 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>39VRVKCF</t>
+          <t>5FPANY5G</t>
         </is>
       </c>
       <c r="C59" s="3" t="n">
-        <v>46237</v>
+        <v>46265</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>B0H54Z8RSJ</t>
+          <t>B0H552PBFY</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>HKNVS25CCBLU</t>
+          <t>HKNVS25CCORG</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -13048,7 +13097,7 @@
         <v>1301</v>
       </c>
       <c r="L59" s="3" t="n">
-        <v>46270</v>
+        <v>46298</v>
       </c>
     </row>
     <row r="60">
@@ -13059,20 +13108,20 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>5FPANY5G</t>
+          <t>39VRVKCF</t>
         </is>
       </c>
       <c r="C60" s="3" t="n">
-        <v>46265</v>
+        <v>46237</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>B0H552PBFY</t>
+          <t>B0H54Z8RSJ</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>HKNVS25CCORG</t>
+          <t>HKNVS25CCBLU</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -13096,7 +13145,7 @@
         <v>1301</v>
       </c>
       <c r="L60" s="3" t="n">
-        <v>46298</v>
+        <v>46270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>